<commit_message>
Kip geçişlerinde köprü, başlıkta en fazla iki konu
- Bir cümle -iyor ile biterken sonraki -mıştır ile başlarsa metin zıplıyor;
  aynı kipteki cümleler yan yana toplanır ya da geçişe köprü ifade konur
- Başlık en fazla iki konu taşır ("Atmosferi, Ses Tasarımı ve Müziği" değil
  "Atmosferi ve Ses Tasarımı")
- "Skor" müzik anlamında kullanılmaz, puanla karışıyor
- BF6 örneğinde atmosfer bölümü yeniden yazıldı, oynanışa takım oyunu ve
  araç dengesi eklendi (1480 kelime)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -536,7 +536,7 @@
 H2: Battlefield 6 Hikâyesi
 H2: Battlefield 6 Oynanışı ve Oyun Modları
 H3: Çok Oyunculu Modlar ve REDSEC
-H2: Battlefield 6 Atmosferi, Ses Tasarımı ve Müziği
+H2: Battlefield 6 Atmosferi ve Ses Tasarımı
 H2: Battlefield 6'da Öne Çıkan Özellikler
 H2: GeForce NOW ile Battlefield 6 Deneyimi
 H3: Battlefield 6'yı GAME+ ile Oynamak
@@ -558,7 +558,7 @@
 H2 · GeForce NOW'da Nasıl Oynanır: Yalnız erişim yanıtı. Oyun kütüphanede mi, hangi mağaza hesabıyla bağlanıyor, kurulum gerekiyor mu, ücretsiz mod varsa şartı ne. Künye bilgisi girişte verildiği için burada tekrarlanmaz.
 H2 · Hikâyesi: Kurulum (hangi yıl, hangi çatışma, kime karşı), oynanan birlik, bölümlerin geçtiği yerler, anlatı biçimi ve doğrulanmış süre. Olay örgüsü, dönüm noktaları ve son yazılmaz.
 H2 · Oynanışı ve Oyun Modları: Hareket ve silah sistemi, sınıflar (madde listesi), araçlar ve yıkım, harita yapısı, geliştirme bağlamı. Alt başlıkta modlar madde listesiyle ve ücretsiz battle royale modu.
-H2 · Atmosferi, Ses Tasarımı ve Müziği: Ton ve sanat tasarımı somut örnekle, ses tasarımı, besteci ve şarkı seçkisi, kazanılan ödüller ile adaylıklar ayrı ayrı.
+H2 · Atmosferi ve Ses Tasarımı: Ton ve sanat tasarımı somut örnekle, ses tasarımı, besteci ve şarkı seçkisi, kazanılan ödüller ile adaylıklar ayrı ayrı.
 H2 · Öne Çıkan Özellikler: Oyunu ayıran başlıklar 6-8 maddelik listede toplanır; bölüm bir cümlelik girişle açılır.
 H2 · GeForce NOW ile Deneyim: Bulutun somut olarak ne değiştirdiği, gecikme, cihaz çeşitliliği, kontrolcü desteği. Alt başlıklarda paketlerin ne sunduğu ve bağlantı hızı tablosu.
 H2 · Sistem Gereksinimleri ve İndirme: PC gereksinimleri tablosu, ardından bulut karşıtlığı. "Bilgisayarım kaldırır mı" burada karşılanır.

</xml_diff>

<commit_message>
Kapanışa Performance / Ultimate paket önerisi (CTA): kurallar, kontrol listesi, BF6 örnekleri, README
Oyuna özel paket gerekliliği yine yazılmıyor; iki paket kapanışta birlikte öneriliyor, fiyat ve paket özelliği yazılmıyor. Örnek brief satırı 30 satır hücre sınırına sığdırıldı.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="409" customHeight="1">
+    <row r="2" ht="396" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Battlefield 6</t>
@@ -553,8 +553,8 @@
               <color rgb="FF10332F"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">TON: Ürün sayfası. Okuyucu ya oyunu tanıyor ve GeForce NOW üzerinden oynayıp oynayamayacağını merak ediyor, ya da oyunu yeni duymuş ve ne olduğuna bakıyor. Her bölüm önce yanıtı verir, açıklama sonra gelir. Kip cümlenin işine göre seçilir: tanım ve kural geniş zaman, kaynaklı veri "-mektedir/-mıştır", anlatı ve atmosfer şimdiki zaman, okuyucuya yönerge ikinci tekil.
-AÇILIŞ: Gövde başlıksız 1-2 paragraflık girişle açılır; oyunu genel olarak tanıtır, puanlar madde listesiyle verilir, resmi dil desteği tek cümleyle belirtilir. Sayfada H1 bulunduğu için bu girişe başlık konmaz. Tür kelimesi ("FPS oyunları") girişte doğal bir cümlenin içinde geçer ve iç link buraya yerleşir.
+            <t>TON: Ürün sayfası. Okuyucu ya oyunu tanıyor ve GeForce NOW'da oynayıp oynayamayacağını merak ediyor, ya da oyunu yeni duymuş. Her bölüm önce yanıtı verir. Kip işe göre: tanım geniş zaman, kaynaklı veri "-mektedir/-mıştır", anlatı şimdiki zaman, yönerge ikinci tekil.
+AÇILIŞ: Başlıksız 1-2 paragraflık giriş (sayfada H1 var); oyunu tanıtır, puanlar madde listesiyle, resmi dil desteği tek cümleyle. Tür kelimesi ("FPS oyunları") girişte doğal bir cümlenin içinde geçer, iç link buraya.
 H2 · GeForce NOW'da Nasıl Oynanır: Yalnız erişim yanıtı. Oyun kütüphanede mi, hangi mağaza hesabıyla bağlanıyor, kurulum gerekiyor mu, ücretsiz mod varsa şartı ne. Künye bilgisi girişte verildiği için burada tekrarlanmaz.
 H2 · Hikâyesi: Kurulum (hangi yıl, hangi çatışma, kime karşı), oynanan birlik, bölümlerin geçtiği yerler, anlatı biçimi ve doğrulanmış süre. Olay örgüsü, dönüm noktaları ve son yazılmaz.
 H2 · Oynanışı ve Oyun Modları: Hareket ve silah sistemi, sınıflar (madde listesi), araçlar ve yıkım, harita yapısı, geliştirme bağlamı. Alt başlıkta modlar madde listesiyle ve ücretsiz battle royale modu.
@@ -564,9 +564,9 @@
 H2 · Sistem Gereksinimleri ve İndirme: PC gereksinimleri tablosu, ardından bulut karşıtlığı. "Bilgisayarım kaldırır mı" burada karşılanır.
 H2 · Ücretsiz mi, Nasıl Başlanır: Erişim modeli, katalogda desteklenen mağazalar ve 3 maddelik numaralı başlama adımları. Bölümün sonunda kısa bir kapanış çağrısı yer alır.
 SSS: Sayfanın ayrı modülünde yer alır ve gövde kelime sayısına dahil değildir.
-BİÇİM: Sınıflar, modlar, puanlar ve öne çıkan özellikler madde listesiyle; bağlantı hızı ve sistem gereksinimleri tabloyla verilir. Önemli terim ve değerler kalın yazılır. İç linkler zaten var olan bir cümlenin içine yerleşir; "şu listeye göz atabilirsin" biçiminde ek cümle kurulmaz.
+BİÇİM: Sınıflar, modlar, puanlar ve öne çıkan özellikler madde listesiyle; bağlantı hızı ve sistem gereksinimleri tabloyla. Önemli terimler kalın. İç link var olan bir cümlenin içine yerleşir, link için ek cümle kurulmaz. Kapanışta bir iki cümleyle oyunu oynamak için Performance ya da Ultimate paketlerinden birinin seçilebileceği söylenip satın almaya çağrılır; fiyat ve paket özelliği yazılmaz.
 UZUNLUK: Ortalama 1200-1500 kelime gövde. Paragraflar en fazla 3-4 cümledir; teknik değerler (GB, Mbps, çözünürlük, süre) rakamla yazılır.
-DİKKAT: Fiyat, indirim ve kampanya bilgisi yazılmaz. Oyunun hangi GAME+ paketiyle oynanabileceği yazılmaz. GFN optimizasyon durumu yazılmaz. Puan, gereksinim, boyut ve dil listesi PC sürümünden alınır. Mağaza listesi katalogdaki variants alanından gelir; oyun başka mağazada satılsa da GFN desteklemiyorsa yazılmaz. Main KW hacminin büyük bölümü çıkış dönemine aittir (Ekim 2025: 135.000, Kasım 2025: 110.000); Mayıs-Temmuz 2026 ortalaması 15.900'dür. </t>
+DİKKAT: Fiyat, indirim ve kampanya bilgisi, oyuna özel paket gerekliliği ve GFN optimizasyon durumu yazılmaz. Puan, gereksinim, boyut ve dil listesi PC sürümünden alınır. Mağaza listesi katalogdaki variants alanından gelir; oyun başka mağazada satılsa da GFN desteklemiyorsa yazılmaz. Main KW hacminin büyük bölümü çıkış dönemine aittir (Ekim 2025: 135.000, Kasım 2025: 110.000); Mayıs-Temmuz 2026 ortalaması 15.900'dür.</t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Türkçe SSS her oyunda, zamandan bağımsız tarih dili, resmi değeri olmayan sayılar için ortalama aralık, düşük puanın korunması
- Türkçe sorusu SSS'de her zaman yer alır; resmi dil değilse 'Hayır' ile yanıtlanır, H2 yalnız resmi destekte
- 'çıkacak/yakında/şu an' yerine tarihli kalıplar ('23 Ekim 2026 çıkış tarihli')
- Kurulum boyutu ve süre için resmi değer yoksa iki kaynaktan ortalama aralık
- Soru biçimi: kullanıcının arattığı ve doğal sözdizimi (brief düzeltmelerinden)
- BF6 örnekleri: Türkçe SSS, 'kampanya' kelimesi temizlendi

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -604,11 +604,11 @@
 3. Battlefield 6 kaç GB?
    Yanıtta: PC kurulum boyutu ve bulut üzerinden oynarken indirme gerekmediği.
 4. Battlefield 6 Türkçe mi?
-   Yanıtta: resmi arayüz ve altyazı desteği durumu.
+   Yanıtta: resmi Türkçe dil desteği olmadığı (arayüz, altyazı ve seslendirme); desteklenen dillerden örnek.
 5. Bilgisayarım Battlefield 6'yı kaldırır mı?
    Yanıtta: PC gereksinimi ile bulut üzerinden oynama arasındaki fark.
 6. Battlefield 6'da hikâye modu var mı, kaç saat sürüyor?
-   Yanıtta: kampanyanın varlığı ve yaklaşık süresi.
+   Yanıtta: hikâye modunun varlığı ve yaklaşık süresi.
 7. Battlefield 6 RedSec nedir, battle royale ücretsiz mi?
    Yanıtta: RedSec'in Battlefield 6 ile ilişkisi ve erişim koşulu.
 8. Battlefield 6 çevrimdışı oynanabilir mi?

</xml_diff>

<commit_message>
Paket bölümü başlığı: "{Oyun}'ı GAME+ GeForce NOW ile Oynamak"
Kullanıcı kararı (28.09.2026): hizmet adı başlıkta tam geçsin. Kurallar,
brief şablonu, kontrol listesi, denetim betiği ve BF6 örnek brief'i
güncellendi. BF6 örnek içeriği onaydan sonra yeni sürümle değişecek.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -538,7 +538,7 @@
 H3: Çok Oyunculu Modlar ve REDSEC
 H2: Battlefield 6 Atmosferi ve Ses Tasarımı
 H2: Battlefield 6'da Öne Çıkan Özellikler
-H2: Battlefield 6'yı GAME+ ile Oynamak
+H2: Battlefield 6'yı GAME+ GeForce NOW ile Oynamak
 H3: Bağlantı Hızı ve Görüntü Kalitesi
 H2: Battlefield 6 Sistem Gereksinimleri ve İndirme
 H2: Battlefield 6 Ücretsiz mi, Nasıl Başlanır?</t>
@@ -559,7 +559,7 @@
 H2 · Oynanışı ve Oyun Modları: Hareket ve silah sistemi, sınıflar (madde listesi), araçlar ve yıkım, harita yapısı, geliştirme bağlamı. Alt başlıkta modlar madde listesiyle ve ücretsiz battle royale modu.
 H2 · Atmosferi ve Ses Tasarımı: Ton ve sanat tasarımı somut örnekle, ses tasarımı, besteci ve şarkı seçkisi, kazanılan ödüller ile adaylıklar ayrı ayrı.
 H2 · Öne Çıkan Özellikler: Oyunu ayıran başlıklar 6-8 maddelik listede toplanır; bölüm bir cümlelik girişle açılır.
-H2 · GAME+ ile Oynamak: Steam ya da EA App hesabıyla açıldığı, satın almış olmanın yeterli olduğu; paketlerin sunduğu değerler anlatılır, gereken paket yazılmaz.
+H2 · GAME+ GeForce NOW ile Oynamak: Steam ya da EA App hesabıyla açıldığı, satın almış olmanın yeterli olduğu; paketlerin sunduğu değerler anlatılır, gereken paket yazılmaz.
 H3 · Bağlantı Hızı ve Görüntü Kalitesi: Önerilen bağlantı hızı tablosu (yayın kalitesi / hız / platform; 720p/60 15, 1080p/60 25, 4K/120 45 Mbps+) ve gecikme notu (80 ms altı, ideal 40 ms); oyunun HDR ve NVIDIA Reflex desteği yazılır.
 H2 · Sistem Gereksinimleri ve İndirme: PC gereksinimleri tablosu, ardından bulut karşıtlığı. "Bilgisayarım kaldırır mı" burada karşılanır.
 H2 · Ücretsiz mi, Nasıl Başlanır: Erişim modeli, katalogda desteklenen mağazalar ve 3 maddelik numaralı başlama adımları. Bölümün sonunda kısa bir kapanış çağrısı yer alır.
@@ -588,7 +588,7 @@
 3. cloud gaming nedir : https://gameplus.com.tr/blog/cloud-gaming-nedir
    H2 · GeForce NOW'da Nasıl Oynanır bölümünün ilk paragrafında.
 4. geforce now paketleri : https://gameplus.com.tr/gfn/paketler
-   H2 · GAME+ ile Oynamak bölümünde, paketlerin anlatıldığı cümlede.
+   H2 · GAME+ GeForce NOW ile Oynamak bölümünde, paketlerin anlatıldığı cümlede.
 5. battlefield 6 sistem gereksinimleri : https://gameplus.com.tr/blog/battlefield-6-incelemesi-fiyat-sistem-gereksinimleri-ilk-yorumlar
    H2 · Sistem Gereksinimleri ve İndirme bölümünde, tablonun altındaki cümlede.
 6. ücretsiz oyunlar : https://gameplus.com.tr/gfn/oyunlar/oynamasi-ucretsiz

</xml_diff>

<commit_message>
Resmi dil desteği GeForce NOW kaydından: brief'e 10. sütun, dil_hucresi.py
Kullanıcı kararı (28.09.2026): resmi dil verisi GeForce NOW'un kendi katalog
dökümünden (gfn_apps_TR.json) alınır.
- scripts/dil_hucresi.py: Türkçe durumu (mağaza ya da katman farkıyla:
  "yalnız Battle.net", "Seslendirme yalnız Xbox") ve tüm mağazalarda ortak
  arayüz / altyazı / seslendirme dilleri; bir mağazadaki fazlalık ayrıca
  yazılır ("Xbox sürümünde +13 dil").
- brief_satiri.py: 10. sütun "Resmi Dil Desteği (GeForce NOW)"; dil alanı
  yoksa hücreyi oyun adından üretir.
- Kurallar: kaynak GFN kaydı, mağaza farkı içerikte yazılır, kayıt eksik
  görünüyorsa (Albion Online) kullanıcıya sorulur.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,7 @@
     <col width="72" customWidth="1" min="7" max="7"/>
     <col width="66" customWidth="1" min="8" max="8"/>
     <col width="58" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -496,6 +497,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Yanıt Biçimi</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Resmi Dil Desteği (GeForce NOW)</t>
         </is>
       </c>
     </row>
@@ -628,6 +634,14 @@
 • Doğrulanamayan bilgi yazılmaz; yanıtlanamayan soru listeden çıkarılır.</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Türkçe: Yok
+Arayüz (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
+Altyazı (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
+Seslendirme (1): İngilizce · Steam sürümünde +10 dil</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Türkçe dil desteği: mağaza birleşimi, menü/altyazı/Türkçe dublaj terimleri, dublaj teyidi
- dil_hucresi.py: Türkçe satırı mağaza sürümlerinin birleşimi; ayrışmada Doğrula notu
- Referanslar ve SKILL.md: içerikte mağaza farkı yazılmaz, dublaj teyitli kaynaktan gelir
- icerik_denetim.py: Türkçe cümlesinde mağaza farkı sorun, arayüz/seslendirme terimi not
- brief_satiri.py: kalın uyarı cümlesi gövdeye boşlukla eklenir
- BF6 örnek brief: Türkçe notu kurala uyduruldu, xlsx yeniden üretildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -581,7 +581,7 @@
               <color rgb="FF10332F"/>
               <sz val="10"/>
             </rPr>
-            <t>Türkçe dil desteği doğrulanamazsa ve resmi, modsuz dil desteği yoksa ilgili H2 ve SSS sorusu çıkarılır.</t>
+            <t xml:space="preserve"> Resmi Türkçe desteği yoktur: ayrı H2 açılmaz, SSS'de "Hayır" ile yanıtlanır.</t>
           </r>
         </is>
       </c>
@@ -610,7 +610,7 @@
 3. Battlefield 6 kaç GB?
    Yanıtta: PC kurulum boyutu ve bulut üzerinden oynarken indirme gerekmediği.
 4. Battlefield 6 Türkçe mi?
-   Yanıtta: resmi Türkçe dil desteği olmadığı (arayüz, altyazı ve seslendirme); desteklenen dillerden örnek.
+   Yanıtta: resmi Türkçe menü, altyazı ve dublaj olmadığı; menü dillerinin sayısı.
 5. Bilgisayarım Battlefield 6'yı kaldırır mı?
    Yanıtta: PC gereksinimi ile bulut üzerinden oynama arasındaki fark.
 6. Battlefield 6'da hikâye modu var mı, kaç saat sürüyor?
@@ -637,9 +637,9 @@
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Türkçe: Yok
-Arayüz (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
+Menü (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
 Altyazı (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
-Seslendirme (1): İngilizce · Steam sürümünde +10 dil</t>
+Seslendirme (1): İngilizce · Steam listesinde +10 dil</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dil desteği: PC listesi esas, her brief'te Steam dil tablosuyla teyit
- dil_teyit.py (yeni): GFN PC sürümleri (Xbox hariç) ile Steam dil tablosunu karşılaştırır, brief satırı önerir
- dil_hucresi.py: PC variantı varken Xbox listesi hesaba katılmaz; teyitsiz hücreye uyarı satırı
- brief_satiri.py: dil_teyit alanı, sütun adı 'Resmi Dil Desteği (PC)'
- dogrulama.md: karar sırası (Steam tablosu > GFN PC kaydı/yayıncı > yayıncı kaynağı), BF1/Overwatch/Fortnite örnekleri
- SKILL.md, brief/içerik kuralları, kontrol listesi, BF6 örneği güncellendi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ornek-brief-battlefield-6.xlsx
+++ b/examples/ornek-brief-battlefield-6.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Resmi Dil Desteği (GeForce NOW)</t>
+          <t>Resmi Dil Desteği (PC)</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Türkçe: Yok
+          <t>Türkçe: Yok (teyit: Steam dil tablosu)
 Menü (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
 Altyazı (13): İngilizce, Fransızca, Almanca, İspanyolca, İspanyolca (Latin Amerika), Çince (Basitleştirilmiş), Çince (Geleneksel), Japonca, İtalyanca, Portekizce (Brezilya), Korece, Lehçe, Arapça
 Seslendirme (1): İngilizce · Steam listesinde +10 dil</t>

</xml_diff>